<commit_message>
feat: add /canonical page, canonical templates engine, and denormalized master taxonomy tables
</commit_message>
<xml_diff>
--- a/docs/PromptCanvas_Architecture_Taxonomy_v1.0_Consolidated.xlsx
+++ b/docs/PromptCanvas_Architecture_Taxonomy_v1.0_Consolidated.xlsx
@@ -3,11 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Architecture Families (39)" sheetId="1" r:id="rId1"/>
-    <sheet name="Visual Grammars (34 Schemas)" sheetId="2" r:id="rId2"/>
-    <sheet name="Visual Families (8)" sheetId="3" r:id="rId3"/>
-    <sheet name="Document Bindings (16)" sheetId="4" r:id="rId4"/>
-    <sheet name="Bio-Pharma Architecture" sheetId="5" r:id="rId5"/>
+    <sheet name="Denormalized Master Matrix (39)" sheetId="1" r:id="rId1"/>
+    <sheet name="Architecture Families (39)" sheetId="2" r:id="rId2"/>
+    <sheet name="Visual Grammars (34 Schemas)" sheetId="3" r:id="rId3"/>
+    <sheet name="Visual Families (8)" sheetId="4" r:id="rId4"/>
+    <sheet name="Document Bindings (16)" sheetId="5" r:id="rId5"/>
+    <sheet name="Bio-Pharma Architecture" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -408,13 +409,13 @@
         <v>seq_no</v>
       </c>
       <c r="B1" t="str">
+        <v>family_id</v>
+      </c>
+      <c r="C1" t="str">
+        <v>family_name</v>
+      </c>
+      <c r="D1" t="str">
         <v>family_type</v>
-      </c>
-      <c r="C1" t="str">
-        <v>family_id</v>
-      </c>
-      <c r="D1" t="str">
-        <v>family_name</v>
       </c>
       <c r="E1" t="str">
         <v>parent_family</v>
@@ -423,37 +424,37 @@
         <v>applicable_levels</v>
       </c>
       <c r="G1" t="str">
-        <v>required_views</v>
+        <v>required_views_denormalized</v>
       </c>
       <c r="H1" t="str">
-        <v>recommended_views</v>
+        <v>recommended_views_denormalized</v>
       </c>
       <c r="I1" t="str">
-        <v>conditional_views</v>
+        <v>conditional_views_denormalized</v>
       </c>
       <c r="J1" t="str">
         <v>variants</v>
       </c>
       <c r="K1" t="str">
-        <v>technology_bindings</v>
+        <v>technology_bindings_gcp_and_oss</v>
       </c>
       <c r="L1" t="str">
-        <v>document_bindings</v>
+        <v>document_bindings_denormalized</v>
       </c>
       <c r="M1" t="str">
-        <v>assurance_framework_version</v>
+        <v>assurance_and_security_standards</v>
       </c>
       <c r="N1" t="str">
-        <v>industry_tags</v>
+        <v>industry_vertical_tags</v>
       </c>
       <c r="O1" t="str">
-        <v>trigger_conditions</v>
+        <v>trigger_conditions_and_intent</v>
       </c>
       <c r="P1" t="str">
-        <v>traceability_relations</v>
+        <v>end_to_end_traceability_flow</v>
       </c>
       <c r="Q1" t="str">
-        <v>description_l1_l2_l3</v>
+        <v>architectural_scope_l1_l2_l3</v>
       </c>
     </row>
     <row r="2">
@@ -461,13 +462,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
+        <v>APP-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Application &amp; Service Architecture</v>
+      </c>
+      <c r="D2" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C2" t="str">
-        <v>APP-01</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Application &amp; Service Architecture</v>
       </c>
       <c r="E2" t="str">
         <v>Application &amp; Services</v>
@@ -514,13 +515,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
+        <v>APP-02</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Serverless &amp; Function-as-a-Service Architecture</v>
+      </c>
+      <c r="D3" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C3" t="str">
-        <v>APP-02</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Serverless &amp; Function-as-a-Service Architecture</v>
       </c>
       <c r="E3" t="str">
         <v>Application &amp; Services</v>
@@ -567,13 +568,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
+        <v>APP-03</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Event-Driven Architecture (EDA) &amp; Async Mesh</v>
+      </c>
+      <c r="D4" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C4" t="str">
-        <v>APP-03</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Event-Driven Architecture (EDA) &amp; Async Mesh</v>
       </c>
       <c r="E4" t="str">
         <v>Application &amp; Services</v>
@@ -620,13 +621,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
+        <v>APP-04</v>
+      </c>
+      <c r="C5" t="str">
+        <v>SaaS Multi-Tenant Architecture &amp; Data Isolation</v>
+      </c>
+      <c r="D5" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C5" t="str">
-        <v>APP-04</v>
-      </c>
-      <c r="D5" t="str">
-        <v>SaaS Multi-Tenant Architecture &amp; Data Isolation</v>
       </c>
       <c r="E5" t="str">
         <v>Application &amp; Services</v>
@@ -673,13 +674,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
+        <v>APP-05</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Enterprise CI/CD &amp; GitOps Software Delivery</v>
+      </c>
+      <c r="D6" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C6" t="str">
-        <v>APP-05</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Enterprise CI/CD &amp; GitOps Software Delivery</v>
       </c>
       <c r="E6" t="str">
         <v>Application &amp; Services</v>
@@ -726,13 +727,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
+        <v>APP-06</v>
+      </c>
+      <c r="C7" t="str">
+        <v>API Platform &amp; Integration Architecture</v>
+      </c>
+      <c r="D7" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C7" t="str">
-        <v>APP-06</v>
-      </c>
-      <c r="D7" t="str">
-        <v>API Platform &amp; Integration Architecture</v>
       </c>
       <c r="E7" t="str">
         <v>Application &amp; Services</v>
@@ -779,13 +780,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
+        <v>APP-07</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Micro-Frontend &amp; Edge SSR Composition</v>
+      </c>
+      <c r="D8" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C8" t="str">
-        <v>APP-07</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Micro-Frontend &amp; Edge SSR Composition</v>
       </c>
       <c r="E8" t="str">
         <v>Application &amp; Services</v>
@@ -832,13 +833,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
+        <v>APP-08</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Enterprise Integration &amp; B2B/EDI Hub</v>
+      </c>
+      <c r="D9" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C9" t="str">
-        <v>APP-08</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Enterprise Integration &amp; B2B/EDI Hub</v>
       </c>
       <c r="E9" t="str">
         <v>Application &amp; Services</v>
@@ -885,13 +886,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
+        <v>CLD-01</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Cloud Foundation &amp; Landing Zone Architecture</v>
+      </c>
+      <c r="D10" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C10" t="str">
-        <v>CLD-01</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Cloud Foundation &amp; Landing Zone Architecture</v>
       </c>
       <c r="E10" t="str">
         <v>Cloud, Network &amp; Infrastructure</v>
@@ -938,13 +939,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
+        <v>CLD-02</v>
+      </c>
+      <c r="C11" t="str">
+        <v>High Availability &amp; Disaster Recovery (HA/DR)</v>
+      </c>
+      <c r="D11" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C11" t="str">
-        <v>CLD-02</v>
-      </c>
-      <c r="D11" t="str">
-        <v>High Availability &amp; Disaster Recovery (HA/DR)</v>
       </c>
       <c r="E11" t="str">
         <v>Cloud, Network &amp; Infrastructure</v>
@@ -991,13 +992,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
+        <v>CLD-03</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Kubernetes &amp; Container Platform Architecture</v>
+      </c>
+      <c r="D12" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C12" t="str">
-        <v>CLD-03</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Kubernetes &amp; Container Platform Architecture</v>
       </c>
       <c r="E12" t="str">
         <v>Cloud, Network &amp; Infrastructure</v>
@@ -1044,13 +1045,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
+        <v>CLD-04</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Hybrid &amp; Multi-Cloud Connectivity Architecture</v>
+      </c>
+      <c r="D13" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C13" t="str">
-        <v>CLD-04</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Hybrid &amp; Multi-Cloud Connectivity Architecture</v>
       </c>
       <c r="E13" t="str">
         <v>Cloud, Network &amp; Infrastructure</v>
@@ -1097,13 +1098,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
+        <v>NET-01</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Private Ingress, Egress &amp; Controlled Connectivity</v>
+      </c>
+      <c r="D14" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C14" t="str">
-        <v>NET-01</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Private Ingress, Egress &amp; Controlled Connectivity</v>
       </c>
       <c r="E14" t="str">
         <v>Cloud, Network &amp; Infrastructure</v>
@@ -1150,13 +1151,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
+        <v>NET-02</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Zero-Trust Network Microsegmentation &amp; Service Mesh</v>
+      </c>
+      <c r="D15" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C15" t="str">
-        <v>NET-02</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Zero-Trust Network Microsegmentation &amp; Service Mesh</v>
       </c>
       <c r="E15" t="str">
         <v>Cloud, Network &amp; Infrastructure</v>
@@ -1203,13 +1204,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
+        <v>DAT-01</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Enterprise Data Platform &amp; Lakehouse</v>
+      </c>
+      <c r="D16" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C16" t="str">
-        <v>DAT-01</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Enterprise Data Platform &amp; Lakehouse</v>
       </c>
       <c r="E16" t="str">
         <v>Data &amp; Analytics</v>
@@ -1256,13 +1257,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
+        <v>DAT-02</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Real-Time Streaming &amp; Event Analytics Pipeline</v>
+      </c>
+      <c r="D17" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C17" t="str">
-        <v>DAT-02</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Real-Time Streaming &amp; Event Analytics Pipeline</v>
       </c>
       <c r="E17" t="str">
         <v>Data &amp; Analytics</v>
@@ -1309,13 +1310,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
+        <v>DAT-03</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Dimensional Data Modeling &amp; Star Schema</v>
+      </c>
+      <c r="D18" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C18" t="str">
-        <v>DAT-03</v>
-      </c>
-      <c r="D18" t="str">
-        <v>Dimensional Data Modeling &amp; Star Schema</v>
       </c>
       <c r="E18" t="str">
         <v>Data &amp; Analytics</v>
@@ -1362,13 +1363,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
+        <v>DAT-04</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Unified Data Governance &amp; Data Mesh</v>
+      </c>
+      <c r="D19" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C19" t="str">
-        <v>DAT-04</v>
-      </c>
-      <c r="D19" t="str">
-        <v>Unified Data Governance &amp; Data Mesh</v>
       </c>
       <c r="E19" t="str">
         <v>Data &amp; Analytics</v>
@@ -1415,13 +1416,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
+        <v>DAT-05</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Data Lineage, Provenance &amp; Quality Lifecycle</v>
+      </c>
+      <c r="D20" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C20" t="str">
-        <v>DAT-05</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Data Lineage, Provenance &amp; Quality Lifecycle</v>
       </c>
       <c r="E20" t="str">
         <v>Data &amp; Analytics</v>
@@ -1468,13 +1469,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
+        <v>DAT-06</v>
+      </c>
+      <c r="C21" t="str">
+        <v>MLOps &amp; Machine Learning Lifecycle Architecture</v>
+      </c>
+      <c r="D21" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C21" t="str">
-        <v>DAT-06</v>
-      </c>
-      <c r="D21" t="str">
-        <v>MLOps &amp; Machine Learning Lifecycle Architecture</v>
       </c>
       <c r="E21" t="str">
         <v>Data &amp; Analytics</v>
@@ -1521,13 +1522,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
+        <v>DAT-07</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Graph Database &amp; Semantic Knowledge Graph</v>
+      </c>
+      <c r="D22" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C22" t="str">
-        <v>DAT-07</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Graph Database &amp; Semantic Knowledge Graph</v>
       </c>
       <c r="E22" t="str">
         <v>Data &amp; Analytics</v>
@@ -1574,13 +1575,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
+        <v>AI-01</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Retrieval-Augmented Generation (RAG) Architecture</v>
+      </c>
+      <c r="D23" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C23" t="str">
-        <v>AI-01</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Retrieval-Augmented Generation (RAG) Architecture</v>
       </c>
       <c r="E23" t="str">
         <v>AI &amp; Cognitive Systems</v>
@@ -1627,13 +1628,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
+        <v>AI-02</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Multi-Agent Systems &amp; Orchestration Architecture</v>
+      </c>
+      <c r="D24" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C24" t="str">
-        <v>AI-02</v>
-      </c>
-      <c r="D24" t="str">
-        <v>Multi-Agent Systems &amp; Orchestration Architecture</v>
       </c>
       <c r="E24" t="str">
         <v>AI &amp; Cognitive Systems</v>
@@ -1680,13 +1681,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
+        <v>AI-03</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Autonomous Agent Tool &amp; Protocol Gateway (MCP / A2A)</v>
+      </c>
+      <c r="D25" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C25" t="str">
-        <v>AI-03</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Autonomous Agent Tool &amp; Protocol Gateway (MCP / A2A)</v>
       </c>
       <c r="E25" t="str">
         <v>AI &amp; Cognitive Systems</v>
@@ -1733,13 +1734,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
+        <v>AI-04</v>
+      </c>
+      <c r="C26" t="str">
+        <v>AI Safety, Guardrails &amp; Evaluation Architecture</v>
+      </c>
+      <c r="D26" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C26" t="str">
-        <v>AI-04</v>
-      </c>
-      <c r="D26" t="str">
-        <v>AI Safety, Guardrails &amp; Evaluation Architecture</v>
       </c>
       <c r="E26" t="str">
         <v>AI &amp; Cognitive Systems</v>
@@ -1786,13 +1787,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
+        <v>AI-05</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Intelligent Document Processing (IDP) Architecture</v>
+      </c>
+      <c r="D27" t="str">
         <v>Solution</v>
-      </c>
-      <c r="C27" t="str">
-        <v>AI-05</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Intelligent Document Processing (IDP) Architecture</v>
       </c>
       <c r="E27" t="str">
         <v>AI &amp; Cognitive Systems</v>
@@ -1839,13 +1840,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
+        <v>AI-06</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Logical AI Tenant Isolation &amp; Context Routing</v>
+      </c>
+      <c r="D28" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C28" t="str">
-        <v>AI-06</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Logical AI Tenant Isolation &amp; Context Routing</v>
       </c>
       <c r="E28" t="str">
         <v>AI &amp; Cognitive Systems</v>
@@ -1892,13 +1893,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
+        <v>SEC-01</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Enterprise Identity, Access &amp; Zero-Trust Architecture</v>
+      </c>
+      <c r="D29" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C29" t="str">
-        <v>SEC-01</v>
-      </c>
-      <c r="D29" t="str">
-        <v>Enterprise Identity, Access &amp; Zero-Trust Architecture</v>
       </c>
       <c r="E29" t="str">
         <v>Security, Privacy &amp; Sovereignty</v>
@@ -1945,13 +1946,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
+        <v>SEC-02</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Application &amp; Workload Security Architecture</v>
+      </c>
+      <c r="D30" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C30" t="str">
-        <v>SEC-02</v>
-      </c>
-      <c r="D30" t="str">
-        <v>Application &amp; Workload Security Architecture</v>
       </c>
       <c r="E30" t="str">
         <v>Security, Privacy &amp; Sovereignty</v>
@@ -1998,13 +1999,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
+        <v>SEC-03</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Threat Modeling &amp; Attack Surface Architecture (STRIDE)</v>
+      </c>
+      <c r="D31" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C31" t="str">
-        <v>SEC-03</v>
-      </c>
-      <c r="D31" t="str">
-        <v>Threat Modeling &amp; Attack Surface Architecture (STRIDE)</v>
       </c>
       <c r="E31" t="str">
         <v>Security, Privacy &amp; Sovereignty</v>
@@ -2051,13 +2052,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
+        <v>SEC-04</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Data Security, Privacy &amp; Sovereign Cloud Architecture</v>
+      </c>
+      <c r="D32" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C32" t="str">
-        <v>SEC-04</v>
-      </c>
-      <c r="D32" t="str">
-        <v>Data Security, Privacy &amp; Sovereign Cloud Architecture</v>
       </c>
       <c r="E32" t="str">
         <v>Security, Privacy &amp; Sovereignty</v>
@@ -2104,13 +2105,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
+        <v>OPS-01</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Enterprise Observability, Telemetry &amp; SRE Architecture</v>
+      </c>
+      <c r="D33" t="str">
         <v>Platform</v>
-      </c>
-      <c r="C33" t="str">
-        <v>OPS-01</v>
-      </c>
-      <c r="D33" t="str">
-        <v>Enterprise Observability, Telemetry &amp; SRE Architecture</v>
       </c>
       <c r="E33" t="str">
         <v>Operations &amp; SRE</v>
@@ -2157,13 +2158,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
+        <v>OPS-02</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Operational Readiness &amp; Go-Live Cutover Runbook</v>
+      </c>
+      <c r="D34" t="str">
         <v>Operational</v>
-      </c>
-      <c r="C34" t="str">
-        <v>OPS-02</v>
-      </c>
-      <c r="D34" t="str">
-        <v>Operational Readiness &amp; Go-Live Cutover Runbook</v>
       </c>
       <c r="E34" t="str">
         <v>Operations &amp; SRE</v>
@@ -2210,13 +2211,13 @@
         <v>34</v>
       </c>
       <c r="B35" t="str">
+        <v>STR-01</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Enterprise Discovery, Assessment &amp; Migration Waves</v>
+      </c>
+      <c r="D35" t="str">
         <v>Operational</v>
-      </c>
-      <c r="C35" t="str">
-        <v>STR-01</v>
-      </c>
-      <c r="D35" t="str">
-        <v>Enterprise Discovery, Assessment &amp; Migration Waves</v>
       </c>
       <c r="E35" t="str">
         <v>Strategic &amp; Operating Models</v>
@@ -2263,13 +2264,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="str">
+        <v>STR-02</v>
+      </c>
+      <c r="C36" t="str">
+        <v>AI Operating Model, Governance &amp; Decision Framework</v>
+      </c>
+      <c r="D36" t="str">
         <v>Operational</v>
-      </c>
-      <c r="C36" t="str">
-        <v>STR-02</v>
-      </c>
-      <c r="D36" t="str">
-        <v>AI Operating Model, Governance &amp; Decision Framework</v>
       </c>
       <c r="E36" t="str">
         <v>Strategic &amp; Operating Models</v>
@@ -2316,13 +2317,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="str">
+        <v>STR-03</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Cloud FinOps &amp; Automated Cost Governance</v>
+      </c>
+      <c r="D37" t="str">
         <v>Operational</v>
-      </c>
-      <c r="C37" t="str">
-        <v>STR-03</v>
-      </c>
-      <c r="D37" t="str">
-        <v>Cloud FinOps &amp; Automated Cost Governance</v>
       </c>
       <c r="E37" t="str">
         <v>Strategic &amp; Operating Models</v>
@@ -2369,13 +2370,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="str">
+        <v>IND-01</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Bio-Pharma Precision Oncology &amp; Regulatory Platform</v>
+      </c>
+      <c r="D38" t="str">
         <v>Industry Accelerator</v>
-      </c>
-      <c r="C38" t="str">
-        <v>IND-01</v>
-      </c>
-      <c r="D38" t="str">
-        <v>Bio-Pharma Precision Oncology &amp; Regulatory Platform</v>
       </c>
       <c r="E38" t="str">
         <v>Industry Accelerators</v>
@@ -2422,13 +2423,13 @@
         <v>38</v>
       </c>
       <c r="B39" t="str">
+        <v>IND-02</v>
+      </c>
+      <c r="C39" t="str">
+        <v>FinTech Autonomous Wealth &amp; Financial Fraud Engine</v>
+      </c>
+      <c r="D39" t="str">
         <v>Industry Accelerator</v>
-      </c>
-      <c r="C39" t="str">
-        <v>IND-02</v>
-      </c>
-      <c r="D39" t="str">
-        <v>FinTech Autonomous Wealth &amp; Financial Fraud Engine</v>
       </c>
       <c r="E39" t="str">
         <v>Industry Accelerators</v>
@@ -2475,13 +2476,13 @@
         <v>39</v>
       </c>
       <c r="B40" t="str">
+        <v>IND-03</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Smart Manufacturing &amp; Industrial IoT Predictive Maintenance</v>
+      </c>
+      <c r="D40" t="str">
         <v>Industry Accelerator</v>
-      </c>
-      <c r="C40" t="str">
-        <v>IND-03</v>
-      </c>
-      <c r="D40" t="str">
-        <v>Smart Manufacturing &amp; Industrial IoT Predictive Maintenance</v>
       </c>
       <c r="E40" t="str">
         <v>Industry Accelerators</v>
@@ -2532,6 +2533,2137 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q40"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>seq_no</v>
+      </c>
+      <c r="B1" t="str">
+        <v>family_type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>family_id</v>
+      </c>
+      <c r="D1" t="str">
+        <v>family_name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>parent_family</v>
+      </c>
+      <c r="F1" t="str">
+        <v>applicable_levels</v>
+      </c>
+      <c r="G1" t="str">
+        <v>required_views</v>
+      </c>
+      <c r="H1" t="str">
+        <v>recommended_views</v>
+      </c>
+      <c r="I1" t="str">
+        <v>conditional_views</v>
+      </c>
+      <c r="J1" t="str">
+        <v>variants</v>
+      </c>
+      <c r="K1" t="str">
+        <v>technology_bindings</v>
+      </c>
+      <c r="L1" t="str">
+        <v>document_bindings</v>
+      </c>
+      <c r="M1" t="str">
+        <v>assurance_framework_version</v>
+      </c>
+      <c r="N1" t="str">
+        <v>industry_tags</v>
+      </c>
+      <c r="O1" t="str">
+        <v>trigger_conditions</v>
+      </c>
+      <c r="P1" t="str">
+        <v>traceability_relations</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>description_l1_l2_l3</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C2" t="str">
+        <v>APP-01</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Application &amp; Service Architecture</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Application &amp; Services</v>
+      </c>
+      <c r="F2" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G2" t="str">
+        <v>01 Context, 07 Container, 08 Component</v>
+      </c>
+      <c r="H2" t="str">
+        <v>09 Data Flow, 11 Sequence, 16 Deployment</v>
+      </c>
+      <c r="I2" t="str">
+        <v>12 State Machine, 28 Failure Flow</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Microservices, Modular Monolith, Hexagonal/Ports &amp; Adapters, Domain-Driven Design (DDD) Services</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Google Cloud Run, GKE Enterprise, Anthos Service Mesh, Eventarc, Cloud Pub/Sub, Cloud Functions</v>
+      </c>
+      <c r="L2" t="str">
+        <v>PRD, FDD, HLD, LLD, SAD, TDD</v>
+      </c>
+      <c r="M2" t="str">
+        <v>OWASP ASVS 4.0.3, CIS Google Cloud Foundations 3.0</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Cross-Industry, Bio-Pharma, FinTech, Retail, Healthcare</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Core application design, service decomposition, modernization from monolith</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Implements PRD Functional Capabilities -&gt; Realized by GKE/Cloud Run workloads -&gt; Verified by E2E Test Suite</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>L1: Domain boundaries &amp; external actors | L2: Service containers, APIs, databases &amp; ingress routing | L3: Class structures, RPC methods, thread pools &amp; connection pools</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C3" t="str">
+        <v>APP-02</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Serverless &amp; Function-as-a-Service Architecture</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Application &amp; Services</v>
+      </c>
+      <c r="F3" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>01 Context, 07 Container, 08 Component</v>
+      </c>
+      <c r="H3" t="str">
+        <v>09 Data Flow, 16 Deployment, 30 FinOps Flow</v>
+      </c>
+      <c r="I3" t="str">
+        <v>11 Sequence, 28 Failure Flow</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Event-Driven Serverless, Stateless Web Microservices, Ephemeral Background Jobs, Async Task Workers</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Cloud Run, Cloud Functions (2nd Gen), Cloud Tasks, Eventarc, Cloud Scheduler</v>
+      </c>
+      <c r="L3" t="str">
+        <v>PRD, FDD, HLD, LLD, Serverless Spec</v>
+      </c>
+      <c r="M3" t="str">
+        <v>CIS GCP Benchmark 3.0, Serverless Security Top 10</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Cross-Industry, Web APIs, Rapid Innovation, SaaS</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Scale-to-zero workloads, bursty traffic patterns, cost-efficient microservices</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Processes Inbound HTTP/Event Triggers -&gt; Scales Ephemeral Containers -&gt; Emits Execution Telemetry</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>L1: Event triggers -&gt; Serverless runtime -&gt; Target storage/APIs | L2: Cloud Run services, concurrency limits, cold-start buffers | L3: Container concurrency (e.g. 80), memory limits (512MB-4GB), vCPU allocations</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C4" t="str">
+        <v>APP-03</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Event-Driven Architecture (EDA) &amp; Async Mesh</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Application &amp; Services</v>
+      </c>
+      <c r="F4" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G4" t="str">
+        <v>09 Data Flow, 10 Integration, 11 Sequence</v>
+      </c>
+      <c r="H4" t="str">
+        <v>08 Component, 16 Deployment, 28 Failure Flow</v>
+      </c>
+      <c r="I4" t="str">
+        <v>12 State Machine, 30 FinOps Flow</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Choreography, Stateful Saga Orchestration, Event Sourcing, Event-Carried State Transfer, Dead-Letter Quarantine</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Cloud Pub/Sub, Eventarc, Cloud Workflows, Cloud Tasks, Cloud Run</v>
+      </c>
+      <c r="L4" t="str">
+        <v>PRD, FDD, HLD, LLD, Async Event Catalog (CloudEvents 1.0)</v>
+      </c>
+      <c r="M4" t="str">
+        <v>CloudEvents 1.0 Specification, Reactive Systems Standard</v>
+      </c>
+      <c r="N4" t="str">
+        <v>FinTech, E-Commerce, Logistics, Real-Time Notifications</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Asynchronous decoupling, high-throughput event brokering, distributed transaction sagas</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Emits Domain Events -&gt; Routes via Pub/Sub Topics -&gt; Compensates on Distributed Failures</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>L1: Event producers -&gt; Enterprise Event Broker -&gt; Decoupled Consumers -&gt; Audit Sink | L2: Pub/Sub topics, Eventarc trigger filters, Workflows saga orchestrator, DLQs | L3: CloudEvents JSON schemas, ack deadline timers, exponential backoff retries</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C5" t="str">
+        <v>APP-04</v>
+      </c>
+      <c r="D5" t="str">
+        <v>SaaS Multi-Tenant Architecture &amp; Data Isolation</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Application &amp; Services</v>
+      </c>
+      <c r="F5" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G5" t="str">
+        <v>01 Context, 07 Container, 18 Trust Boundary</v>
+      </c>
+      <c r="H5" t="str">
+        <v>08 Component, 14 Data Model, 30 FinOps Flow</v>
+      </c>
+      <c r="I5" t="str">
+        <v>17 IAM Flow, 28 Failure Flow</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Silo Model (Dedicated Compute/DB), Pool Model (Shared Compute/DB with RLS), Hybrid Bridge Model, Dynamic Tenant Context Propagator</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Cloud Run, GKE Enterprise, Cloud Spanner Multi-Tenant DBs, Cloud SQL with RLS, Apigee X</v>
+      </c>
+      <c r="L5" t="str">
+        <v>PRD, FDD, HLD, LLD, Multi-Tenancy Architecture Spec</v>
+      </c>
+      <c r="M5" t="str">
+        <v>ISO 27001 Multi-Tenancy Controls, SOC 2 Type II Privacy Controls</v>
+      </c>
+      <c r="N5" t="str">
+        <v>SaaS, B2B Enterprise Software, Multi-Tenant Platforms</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Multi-tenant SaaS products, customer data isolation, tier-based tenant metering</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Authenticates Tenant JWT -&gt; Propagates Tenant Context -&gt; Enforces Database RLS &amp; Compute Quotas</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>L1: Tenant Tiers (Free/Pro/Enterprise) -&gt; Tenant Gateway -&gt; Shared/Isolated Workloads | L2: Tenant routing proxy, tenant context propagator, database RLS policies, tenant billing | L3: Tenant ID schema columns, Redis key namespaces (`tenant:{id}:*`), CPU/RAM hard quotas</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C6" t="str">
+        <v>APP-05</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Enterprise CI/CD &amp; GitOps Software Delivery</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Application &amp; Services</v>
+      </c>
+      <c r="F6" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G6" t="str">
+        <v>20 CI/CD Pipeline, 16 Deployment, 08 Component</v>
+      </c>
+      <c r="H6" t="str">
+        <v>18 Trust Boundary, 21 Observability, 28 Failure Flow</v>
+      </c>
+      <c r="I6" t="str">
+        <v>12 State Machine, 29 Cutover Runbook</v>
+      </c>
+      <c r="J6" t="str">
+        <v>GitOps Declarative Delivery, Trunk-Based Continuous Delivery, Multi-Environment Progressive Delivery (Canary/Blue-Green), Immutable Infrastructure</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Google Cloud Deploy, Cloud Build, Config Sync (GitOps), Artifact Registry, GitHub Actions Enterprise, Prometheus</v>
+      </c>
+      <c r="L6" t="str">
+        <v>HLD, LLD, CI/CD Specification, Release Engineering Guide</v>
+      </c>
+      <c r="M6" t="str">
+        <v>SLSA Framework Level 3, DORA Core Metrics Standard</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Cross-Industry, High-Velocity Software Delivery, Regulated DevOps</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Automated release management, declarative GitOps clusters, progressive canary delivery</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Transforms Git Commits to Verified Container Artifacts -&gt; Progressively Deploys across Dev/Staging/Prod -&gt; Rollback on SLO Alerts</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>L1: Git Repository -&gt; CI Automated Build &amp; Test -&gt; Secure Artifact Store -&gt; CD Pipeline -&gt; Production | L2: Cloud Build pipelines, Artifact Registry vulnerability scanning, Cloud Deploy targets, Config Sync GitOps | L3: Cloud Deploy pipeline phases, canary traffic percentages (10% -&gt; 50% -&gt; 100%), automated verification hooks</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C7" t="str">
+        <v>APP-06</v>
+      </c>
+      <c r="D7" t="str">
+        <v>API Platform &amp; Integration Architecture</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Application &amp; Services</v>
+      </c>
+      <c r="F7" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G7" t="str">
+        <v>01 Context, 10 Integration, 11 Sequence</v>
+      </c>
+      <c r="H7" t="str">
+        <v>08 Component, 17 IAM Flow, 18 Trust Boundary</v>
+      </c>
+      <c r="I7" t="str">
+        <v>25 Tool/Protocol, 30 FinOps Flow</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Enterprise API Gateway, Partner B2B Mesh, Internal Service Mesh Ingress, GraphQL Federation, Async Event Gateway</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Apigee X, Cloud Armor WAF, Global External HTTPS LB, Kong Enterprise, Cloud CDN</v>
+      </c>
+      <c r="L7" t="str">
+        <v>PRD, FDD, HLD, LLD, Security Design, OpenAPI 3.1 Spec</v>
+      </c>
+      <c r="M7" t="str">
+        <v>OWASP API Security Top 10 2023, OAuth 2.1 / OIDC Core 1.0</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Cross-Industry, Open Banking, FHIR Healthcare, B2B Supply Chain</v>
+      </c>
+      <c r="O7" t="str">
+        <v>API lifecycle, external partner exposure, API monetization, microservices mediation</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Exposes Business Capabilities -&gt; Mediated by Apigee X Policies -&gt; Traced via Cloud Trace &amp; Apigee Analytics</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>L1: Consumers -&gt; APIs -&gt; Enterprise capabilities | L2: Gateway, API products, routing, auth, throttling, developer portal | L3: Apigee policies, OAuth2 scopes, quota buckets, XML/JSON transforms, mTLS</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C8" t="str">
+        <v>APP-07</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Micro-Frontend &amp; Edge SSR Composition</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Application &amp; Services</v>
+      </c>
+      <c r="F8" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G8" t="str">
+        <v>01 Context, 07 Container, 08 Component</v>
+      </c>
+      <c r="H8" t="str">
+        <v>10 Integration, 16 Deployment, 21 Observability</v>
+      </c>
+      <c r="I8" t="str">
+        <v>11 Sequence, 30 FinOps Flow</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Module Federation Host Shell, Edge SSR Composition, Web Components, Micro-Apps</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Cloud CDN, Cloud Run Edge SSR, Global HTTPS LB, React / Next.js, Memorystore Redis</v>
+      </c>
+      <c r="L8" t="str">
+        <v>PRD, FDD, HLD, LLD, UX Architecture Spec</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Core Web Vitals Standard, W3C Web Components</v>
+      </c>
+      <c r="N8" t="str">
+        <v>E-Commerce, Portals, SaaS Workspaces, Multi-Team Frontends</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Multi-team frontend scaling, independent frontend deployments, edge page rendering</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Composes Independent Micro-Frontends into Host Shell -&gt; Renders at Edge with Sub-second FCP -&gt; Cached at Cloud CDN</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>L1: Multi-channel user touchpoints &amp; shell boundary | L2: Edge CDN caching, SSR container pods (Nav, Catalog, Checkout), BFF layer | L3: Webpack Module Federation remotes, client state stores, hydration lifecycle</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C9" t="str">
+        <v>APP-08</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Enterprise Integration &amp; B2B/EDI Hub</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Application &amp; Services</v>
+      </c>
+      <c r="F9" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G9" t="str">
+        <v>01 Context, 10 Integration, 09 Data Flow</v>
+      </c>
+      <c r="H9" t="str">
+        <v>08 Component, 16 Deployment, 28 Failure Flow</v>
+      </c>
+      <c r="I9" t="str">
+        <v>11 Sequence, 14 Data Model</v>
+      </c>
+      <c r="J9" t="str">
+        <v>B2B Partner Gateway, EDI X12 / EDIFACT Translator, AS2 / SFTP Managed Transfer, Enterprise Application Integration (EAI)</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Application Integration, Integration Connectors, Cloud Storage SFTP, Apigee X B2B, Cloud Pub/Sub</v>
+      </c>
+      <c r="L9" t="str">
+        <v>HLD, LLD, Partner Integration Spec, EDI Mapping Matrix</v>
+      </c>
+      <c r="M9" t="str">
+        <v>AS2 / RFC 4130 Standard, EDI X12 Standard, ISO 27001</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Supply Chain, Retail Logistics, Healthcare Claims, Manufacturing</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Legacy ERP integration, trading partner EDI communications, managed file transfers</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Receives Inbound B2B EDI Files -&gt; Translates to Canonical JSON Schemas -&gt; Integrates with Core SAP/Oracle ERP</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>L1: External trading partners -&gt; Managed B2B Gateway -&gt; Integration Connectors -&gt; Core Enterprise Systems | L2: Application Integration visual workflows, EDI mapping engines, SFTP buckets, Pub/Sub event queues | L3: EDI X12 segment parsers (850 PO, 810 Invoice), MDN receipt verifiers, AS2 cert exchanges</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C10" t="str">
+        <v>CLD-01</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Cloud Foundation &amp; Landing Zone Architecture</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Cloud, Network &amp; Infrastructure</v>
+      </c>
+      <c r="F10" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G10" t="str">
+        <v>15 Network Topology, 17 IAM Flow, 18 Trust Boundary</v>
+      </c>
+      <c r="H10" t="str">
+        <v>16 Deployment, 21 Observability, 34 Geographic</v>
+      </c>
+      <c r="I10" t="str">
+        <v>19 HA/DR, 30 FinOps Flow</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Hub-and-Spoke VPC, Shared VPC, Multi-Account/Multi-Project Org Hierarchy, Organization Resource Hierarchy</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Google Cloud Organizations, Cloud Router HA, Network Connectivity Center, Resource Manager Folders</v>
+      </c>
+      <c r="L10" t="str">
+        <v>HLD, LLD, Landing Zone Spec, IAM Baseline, Network Architecture Spec</v>
+      </c>
+      <c r="M10" t="str">
+        <v>CIS Google Cloud Benchmark v3.0, NIST SP 800-53 Rev 5</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Cross-Industry, Enterprise Regulated, Sovereign Cloud</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Greenfield GCP onboarding, enterprise landing zone build, multi-tenant cloud organization</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Governs Org Resource Hierarchy -&gt; Enforces Org Policies -&gt; Audited via Cloud Logging &amp; Security Command Center</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>L1: Enterprise organization hierarchy, root folders &amp; cloud boundary | L2: Hub VPC, Spoke VPCs, Shared VPC hosts, interconnects &amp; firewall policies | L3: Subnet CIDRs, BGP ASN routes, resource folders, hierarchical policy bindings</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C11" t="str">
+        <v>CLD-02</v>
+      </c>
+      <c r="D11" t="str">
+        <v>High Availability &amp; Disaster Recovery (HA/DR)</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Cloud, Network &amp; Infrastructure</v>
+      </c>
+      <c r="F11" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G11" t="str">
+        <v>19 HA/DR Architecture, 15 Network Topology, 34 Geographic</v>
+      </c>
+      <c r="H11" t="str">
+        <v>16 Deployment, 21 Observability, 29 Cutover Runbook</v>
+      </c>
+      <c r="I11" t="str">
+        <v>12 State Machine, 28 Failure Flow</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Active-Active Multi-Region, Active-Passive (Hot Standby), Warm Standby, Pilot Light, Backup &amp; Cold Restore</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Cloud Spanner Multi-Region TrueTime, Global External HTTPS LB, Cloud DNS Failover Routing, Cloud Storage Dual-Region Buckets</v>
+      </c>
+      <c r="L11" t="str">
+        <v>HLD, LLD, BCDR Plan, Runbook, Operational Architecture Document (OAD)</v>
+      </c>
+      <c r="M11" t="str">
+        <v>ISO 22301 Business Continuity, NIST SP 800-34 Rev 1</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Banking, Healthcare, Mission-Critical Enterprise, SaaS</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Strict RTO/RPO requirements, multi-region compliance, mission-critical resiliency</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Guarantees SLA/SLO (99.999%) -&gt; Implements Multi-Region Replication -&gt; Validated via Chaos Engineering &amp; Game Days</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>L1: Global geographic regions, failover domains &amp; RTO/RPO targets | L2: Multi-region active-active topology, synchronous DB replication, health-check failover | L3: DNS TTL weights, quorum consensus, cross-region VPC peering &amp; snapshot schedules</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C12" t="str">
+        <v>CLD-03</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Kubernetes &amp; Container Platform Architecture</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Cloud, Network &amp; Infrastructure</v>
+      </c>
+      <c r="F12" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G12" t="str">
+        <v>07 Container, 08 Component, 16 Deployment</v>
+      </c>
+      <c r="H12" t="str">
+        <v>15 Network Topology, 17 IAM Flow, 21 Observability</v>
+      </c>
+      <c r="I12" t="str">
+        <v>19 HA/DR, 20 CI/CD Pipeline</v>
+      </c>
+      <c r="J12" t="str">
+        <v>GKE Autopilot, GKE Enterprise Multi-Cluster Fleet, Anthos Hybrid Cloud, Multi-Tenant Namespaces with Network Policies</v>
+      </c>
+      <c r="K12" t="str">
+        <v>GKE Enterprise, Cilium CNI, Cloud Service Mesh (Istio), Workload Identity Federation, Artifact Registry, Config Sync</v>
+      </c>
+      <c r="L12" t="str">
+        <v>HLD, LLD, Container Platform Blueprint, Security Hardening Guide</v>
+      </c>
+      <c r="M12" t="str">
+        <v>CIS Kubernetes Benchmark v1.8, NIST SP 800-190</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Cross-Industry, Microservices, Cloud Native Platform Engineering</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Containerized workloads, Kubernetes cluster engineering, enterprise platform engineering</v>
+      </c>
+      <c r="P12" t="str">
+        <v>Hosts Application Services -&gt; Enforces Pod Security Standards -&gt; Managed via GitOps Config Sync</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>L1: Enterprise GKE fleet, control planes &amp; multi-region cluster nodes | L2: Namespaces, Ingress controllers, Service Mesh sidecars, Node pools &amp; Workload Identity | L3: HPA/VPA autoscaling, pod disruption budgets, taint/tolerations, Calico network policies</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C13" t="str">
+        <v>CLD-04</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Hybrid &amp; Multi-Cloud Connectivity Architecture</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Cloud, Network &amp; Infrastructure</v>
+      </c>
+      <c r="F13" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G13" t="str">
+        <v>15 Network Topology, 18 Trust Boundary, 34 Geographic</v>
+      </c>
+      <c r="H13" t="str">
+        <v>16 Deployment, 10 Integration, 21 Observability</v>
+      </c>
+      <c r="I13" t="str">
+        <v>19 HA/DR, 30 FinOps Flow</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Dedicated Interconnect (100G/10G), Partner Interconnect, Cross-Cloud Interconnect (AWS/Azure), HA VPN with Cloud Router</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Cloud Interconnect, Cross-Cloud Interconnect (AWS/Azure), Cloud VPN, Cloud Router, Network Connectivity Center (NCC)</v>
+      </c>
+      <c r="L13" t="str">
+        <v>HLD, LLD, Hybrid Network Architecture Spec, BGP Routing Guide</v>
+      </c>
+      <c r="M13" t="str">
+        <v>CIS GCP Foundations 3.0, RFC 4271 BGP-4 Standard</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Multi-Cloud Enterprises, Hybrid Datacenters, Telecommunications</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Connecting on-premises datacenters to GCP, low-latency AWS-to-GCP interconnects, redundant SLA routing</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Establishes Dedicated Fiber Links -&gt; Exchanges Dynamic BGP Routes -&gt; Secures Private High-Bandwidth Cloud Transit</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>L1: On-prem datacenter / AWS / Azure -&gt; Dedicated Interconnect -&gt; Google Cloud Global Backbone | L2: Interconnect attachments (VLANs), Cloud Router BGP active/standby pairs, NCC mesh | L3: BGP ASN 16550 configs, BGP MD5 auth keys, bidirectional forwarding detection (BFD)</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C14" t="str">
+        <v>NET-01</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Private Ingress, Egress &amp; Controlled Connectivity</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Cloud, Network &amp; Infrastructure</v>
+      </c>
+      <c r="F14" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G14" t="str">
+        <v>15 Network Topology, 18 Trust Boundary, 16 Deployment</v>
+      </c>
+      <c r="H14" t="str">
+        <v>01 Context, 19 HA/DR, 34 Geographic</v>
+      </c>
+      <c r="I14" t="str">
+        <v>21 Observability, 28 Failure Flow</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Private Service Connect (PSC) Endpoints, Cloud NAT Static Egress IPs, Cloud DNS Firewall Policies, Direct VPC Egress</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Private Service Connect (PSC), Cloud NAT, Cloud DNS Firewall, Internal Application Load Balancer, Network Security Groups</v>
+      </c>
+      <c r="L14" t="str">
+        <v>HLD, LLD, Network Security &amp; Egress Spec, IP Addressing Plan</v>
+      </c>
+      <c r="M14" t="str">
+        <v>CIS GCP Benchmark v3.0, NIST SP 800-53 (AC-4 Information Flow Enforcement)</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Banking, Healthcare, Regulated Cloud Networks</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Private zero-external-IP architecture, controlled outbound NAT whitelisting, SaaS PSC transit</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Connects Workloads via Private IPs -&gt; Inspects Egress Traffic -&gt; Blocks Unauthorized External Destinations</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>L1: Consumer VPCs -&gt; Private Service Connect -&gt; Managed Producer Services -&gt; Controlled Outbound NAT | L2: PSC forwarding rules, Cloud NAT gateway IP pools, Cloud DNS response policies | L3: Subnet NAT port reservation quotas (min=64, max=1024), PSC attachment URIs, DNS domain blocklists</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C15" t="str">
+        <v>NET-02</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Zero-Trust Network Microsegmentation &amp; Service Mesh</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Cloud, Network &amp; Infrastructure</v>
+      </c>
+      <c r="F15" t="str">
+        <v>L2, L3</v>
+      </c>
+      <c r="G15" t="str">
+        <v>15 Network Topology, 07 Container, 18 Trust Boundary</v>
+      </c>
+      <c r="H15" t="str">
+        <v>08 Component, 21 Observability, 27 Threat Model</v>
+      </c>
+      <c r="I15" t="str">
+        <v>11 Sequence, 17 IAM Flow</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Istio / Cloud Service Mesh mTLS 1.3 Strict Mode, Cilium eBPF Network Policies, Distributed Cloud Firewalls, Ingress/Egress Gateways</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Cloud Service Mesh, Cilium CNI, Hierarchical Firewall Policies, Envoy Proxy, Istio AuthorizationPolicy</v>
+      </c>
+      <c r="L15" t="str">
+        <v>HLD, LLD, Microsegmentation Policy Spec, Service Mesh Blueprint</v>
+      </c>
+      <c r="M15" t="str">
+        <v>NIST SP 800-207 (Zero Trust Architecture), CISA Zero Trust Maturity Model 2.0</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Microservices, PCI-DSS Scoped Environments, Multi-Tenant Platforms</v>
+      </c>
+      <c r="O15" t="str">
+        <v>East-west traffic encryption, service-to-service cryptographic authorization, zero-trust network compliance</v>
+      </c>
+      <c r="P15" t="str">
+        <v>Enforces Cryptographic Pod Identity -&gt; Restricts East-West RPCs -&gt; Audits Network Microsegmentation Logs</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>L1: Microservices mesh boundary with strict mutual cryptographic authentication | L2: Service mesh control plane, Envoy sidecar proxies, ingress/egress gateways, namespace boundaries | L3: AuthorizationPolicy custom resources, PeerAuthentication mTLS strict mode, Cilium eBPF network rules</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C16" t="str">
+        <v>DAT-01</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Enterprise Data Platform &amp; Lakehouse</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Data &amp; Analytics</v>
+      </c>
+      <c r="F16" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G16" t="str">
+        <v>09 Data Flow, 14 Data Model / ERD, 07 Container</v>
+      </c>
+      <c r="H16" t="str">
+        <v>08 Component, 16 Deployment, 30 FinOps Flow</v>
+      </c>
+      <c r="I16" t="str">
+        <v>18 Trust Boundary, 34 Geographic</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Medallion Data Lakehouse (Bronze/Silver/Gold), Data Mesh (Domain-Oriented), Enterprise Data Warehouse (EDW), Hybrid Data Fabric</v>
+      </c>
+      <c r="K16" t="str">
+        <v>BigQuery, Cloud Storage Lake, Dataproc Serverless (Spark), Dataflow (Apache Beam), Dataplex Universal Catalog, Looker</v>
+      </c>
+      <c r="L16" t="str">
+        <v>PRD, FDD, HLD, LLD, Data Architecture Spec, Data Dictionary</v>
+      </c>
+      <c r="M16" t="str">
+        <v>DAMA-DMBOK2, ISO/IEC 38505 Data Governance, GDPR/HIPAA</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Cross-Industry, Healthcare Genomics, Retail Analytics, Financial Data</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Data platform modernization, batch/streaming analytics, enterprise single source of truth</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Ingests Enterprise Raw Data -&gt; Transforms to Conformed Gold Data Marts -&gt; Serves Executive BI &amp; AI Agents</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>L1: Source systems -&gt; Raw Landing -&gt; Curated Conformed -&gt; Analytical Serving -&gt; Consumers | L2: Cloud Storage Bronze, Dataflow ETL, BigQuery Silver/Gold, Dataplex mesh zones | L3: Partitioning/Clustering keys, SCD Type-2 schemas, SQLX transforms, IAM policy tags</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C17" t="str">
+        <v>DAT-02</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Real-Time Streaming &amp; Event Analytics Pipeline</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Data &amp; Analytics</v>
+      </c>
+      <c r="F17" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G17" t="str">
+        <v>09 Data Flow, 10 Integration, 11 Sequence</v>
+      </c>
+      <c r="H17" t="str">
+        <v>08 Component, 16 Deployment, 21 Observability</v>
+      </c>
+      <c r="I17" t="str">
+        <v>28 Failure / Exception Flow</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Sub-second Streaming Analytics, Kappa Architecture, Real-Time Change Data Capture (CDC), Event Sourcing &amp; CQRS</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Cloud Pub/Sub, Datastream CDC, Cloud Dataflow (Apache Beam Streaming), BigQuery Continuous Queries, Memorystore Redis</v>
+      </c>
+      <c r="L17" t="str">
+        <v>PRD, FDD, HLD, LLD, Event Schema Spec (Avro/Protobuf)</v>
+      </c>
+      <c r="M17" t="str">
+        <v>ISO 27001, SOC 2 Type II, FedRAMP High</v>
+      </c>
+      <c r="N17" t="str">
+        <v>FinTech High Frequency, IoT Telemetry, E-Commerce Clickstreams, Real-Time Fraud</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Low-latency data processing, streaming event pipelines, real-time fraud detection</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Consumes Real-time Event Streams -&gt; Processes with Sliding Windows -&gt; Emits Low-Latency Insights to Dashboards &amp; Agents</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>L1: Event producers -&gt; Streaming ingestion -&gt; In-flight stream processing -&gt; Hot/Warm storage -&gt; Real-time actions | L2: Pub/Sub topics, Dataflow streaming pipelines, BigQuery continuous queries, Redis real-time cache | L3: Watermark heuristics, exactly-once processing triggers, dead-letter topics, stateful DoFn buffers</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C18" t="str">
+        <v>DAT-03</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Dimensional Data Modeling &amp; Star Schema</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Data &amp; Analytics</v>
+      </c>
+      <c r="F18" t="str">
+        <v>L2, L3</v>
+      </c>
+      <c r="G18" t="str">
+        <v>14 Data Model / ERD, 08 Component, 09 Data Flow</v>
+      </c>
+      <c r="H18" t="str">
+        <v>07 Container, 30 FinOps Flow, 31 Dependency Map</v>
+      </c>
+      <c r="I18" t="str">
+        <v>18 Trust Boundary, 33 Matrix / Heatmap</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Kimball Star Schema, Snowflake Schema, One Big Table (OBT), Data Vault 2.0</v>
+      </c>
+      <c r="K18" t="str">
+        <v>BigQuery BI Engine, Dataform, dbt Enterprise, BigQuery Materialized Views</v>
+      </c>
+      <c r="L18" t="str">
+        <v>HLD, LLD, Data Warehouse Schema Design, ETL Mapping Spec</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Kimball Dimensional Modeling Methodology</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Cross-Industry, Business Intelligence, Data Warehousing</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Enterprise BI reporting, dimensional data warehouse design, fast BI query caching</v>
+      </c>
+      <c r="P18" t="str">
+        <v>Models Business Metrics into Fact Tables -&gt; Normalizes Conformed Dimensions -&gt; Accelerates Queries via BI Engine</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>L1: Analytical subject marts (Sales, Finance, Inventory) | L2: Fact tables, dimension tables (SCD Type 1/2/3), surrogate keys &amp; grain definitions | L3: Column types, BigQuery physical partitioning by DATE, clustering by composite keys</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C19" t="str">
+        <v>DAT-04</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Unified Data Governance &amp; Data Mesh</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Data &amp; Analytics</v>
+      </c>
+      <c r="F19" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G19" t="str">
+        <v>01 Context, 09 Data Flow, 18 Trust Boundary</v>
+      </c>
+      <c r="H19" t="str">
+        <v>02 Capability Map, 14 Data Model, 34 Geographic</v>
+      </c>
+      <c r="I19" t="str">
+        <v>26 HITL Flow, 30 FinOps Flow</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Decentralized Domain Data Products, Central Governance Mesh, Federated Computational Governance, Data Clean Rooms</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Dataplex Universal Catalog, Sensitive Data Protection (DLP), BigQuery Authorized Views, Analytics Hub</v>
+      </c>
+      <c r="L19" t="str">
+        <v>HLD, LLD, Data Governance Charter, Data Quality SLA Spec</v>
+      </c>
+      <c r="M19" t="str">
+        <v>DAMA-DMBOK2, ISO 8000 Data Quality, EU GDPR</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Cross-Industry, Healthcare Data, Financial Mesh, Retail Sharing</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Cross-domain data sharing, data catalog discovery, automated PII masking and classification</v>
+      </c>
+      <c r="P19" t="str">
+        <v>Catalogs Domain Data Products -&gt; Enforces Fine-Grained Policy Tags -&gt; Audits Data Access in Real-Time</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>L1: Domain data products (Customer, Finance, Supply Chain) -&gt; Universal Catalog -&gt; Mesh Sharing | L2: Dataplex policy tags, fine-grained RLS/CLS masking, automated DLP profiler, Clean Rooms | L3: DLP regex infoTypes, BigQuery dynamic row-level filter expressions, metadata sync jobs</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C20" t="str">
+        <v>DAT-05</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Data Lineage, Provenance &amp; Quality Lifecycle</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Data &amp; Analytics</v>
+      </c>
+      <c r="F20" t="str">
+        <v>L2, L3</v>
+      </c>
+      <c r="G20" t="str">
+        <v>09 Data Flow, 31 Dependency Map, 08 Component</v>
+      </c>
+      <c r="H20" t="str">
+        <v>21 Observability, 28 Failure Flow, 14 Data Model</v>
+      </c>
+      <c r="I20" t="str">
+        <v>18 Trust Boundary, 33 Matrix / Heatmap</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Column-Level Automated Lineage, Data Quality Scorecards, Anomaly Detection at Ingest, Audit Trail Provenance</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Dataplex Data Lineage, Cloud Data Loss Prevention, Dataform Data Quality Assertions, Cloud Logging</v>
+      </c>
+      <c r="L20" t="str">
+        <v>HLD, LLD, Data Quality Framework, Compliance Audit Pack</v>
+      </c>
+      <c r="M20" t="str">
+        <v>ISO 25012 Data Quality, BCBS 239 Risk Data Aggregation</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Banking Regulatory Reporting, Healthcare Clinical Trials, Life Sciences</v>
+      </c>
+      <c r="O20" t="str">
+        <v>Regulatory compliance for data lineage, root-cause debugging of bad data, automated quality scoring</v>
+      </c>
+      <c r="P20" t="str">
+        <v>Traces Data Lineage from Source to Report -&gt; Validates Data Quality Rules -&gt; Alerts on Metric Anomalies</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>L1: End-to-end data lifecycle from operational source to executive report | L2: Column-level lineage graphs, automated quality assertion checkpoints, quarantine queues | L3: OpenLineage JSON schemas, Dataform assertion SQL scripts, quality failure alert webhooks</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C21" t="str">
+        <v>DAT-06</v>
+      </c>
+      <c r="D21" t="str">
+        <v>MLOps &amp; Machine Learning Lifecycle Architecture</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Data &amp; Analytics</v>
+      </c>
+      <c r="F21" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G21" t="str">
+        <v>09 Data Flow, 20 CI/CD Pipeline, 08 Component</v>
+      </c>
+      <c r="H21" t="str">
+        <v>16 Deployment, 21 Observability, 14 Data Model</v>
+      </c>
+      <c r="I21" t="str">
+        <v>28 Failure Flow, 30 FinOps Flow</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Continuous Training (CT) Pipeline, Feature Store Centric, Model Registry &amp; Canary Serving, Distributed GPU/TPU Training</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Vertex AI Pipelines (Kubeflow), Vertex Feature Store, Vertex Model Registry, Vertex Endpoints, BigQuery ML, Cloud TPU v5e</v>
+      </c>
+      <c r="L21" t="str">
+        <v>HLD, LLD, Model Card, AI System Spec, Validation Report</v>
+      </c>
+      <c r="M21" t="str">
+        <v>NIST AI RMF 1.0 (MAP/MEASURE/MANAGE), Google Responsible AI Best Practices</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Bio-Pharma Drug Discovery, Predictive Maintenance, Risk Scoring, Computer Vision</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Production ML models, automated continuous retraining, feature store governance, model registry</v>
+      </c>
+      <c r="P21" t="str">
+        <v>Trains Model Artifacts from Gold Features -&gt; Registers in Model Registry -&gt; Deploys to Scalable Inference Endpoints with Drift Monitoring</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>L1: Feature engineering -&gt; Training -&gt; Evaluation -&gt; Model Registry -&gt; Online/Batch Serving -&gt; Drift Feedback | L2: Vertex AI Pipelines, Kubeflow DAGs, Feature Store, Model Registry, Canary Endpoints | L3: Hyperparameter tuning configs, MLflow metadata artifacts, drift alert thresholds, GPU slice provisioning</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C22" t="str">
+        <v>DAT-07</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Graph Database &amp; Semantic Knowledge Graph</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Data &amp; Analytics</v>
+      </c>
+      <c r="F22" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G22" t="str">
+        <v>14 Data Model / ERD, 09 Data Flow, 08 Component</v>
+      </c>
+      <c r="H22" t="str">
+        <v>24 RAG Flow, 31 Dependency Map, 16 Deployment</v>
+      </c>
+      <c r="I22" t="str">
+        <v>11 Sequence, 18 Trust Boundary</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Property Graph (ISO GQL Standard), Semantic RDF Triple Store, Graph Neural Networks (GNN), Knowledge Graph Multi-Hop</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Cloud Spanner Graph (ISO GQL), Neo4j Enterprise on GCP, Vertex AI Embeddings, BigQuery Graph Analytics</v>
+      </c>
+      <c r="L22" t="str">
+        <v>HLD, LLD, Graph Ontology Specification, Graph Schema Design</v>
+      </c>
+      <c r="M22" t="str">
+        <v>ISO/IEC 39075:2024 (Database Language GQL), W3C RDF/OWL Standards</v>
+      </c>
+      <c r="N22" t="str">
+        <v>Bio-Pharma Genomics, Fraud Rings, Enterprise Knowledge Graphs, Supply Chain</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Complex multi-hop relationships, fraud network detection, biomedical entity linking, GraphRAG reasoning</v>
+      </c>
+      <c r="P22" t="str">
+        <v>Extracts Entities &amp; Relationships -&gt; Builds Graph Nodes &amp; Edges in Spanner Graph -&gt; Executes ISO GQL Multi-Hop Queries</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>L1: Entity domains (Patients, Genes, Diseases, Trials) -&gt; Graph Knowledge Store -&gt; Semantic Query Engine | L2: Graph node labels, edge relationship types, property schemas, graph indexers | L3: ISO GQL MATCH queries, graph partitioning across Spanner splits, GraphRAG traversal depth limits (k=3)</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C23" t="str">
+        <v>AI-01</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Retrieval-Augmented Generation (RAG) Architecture</v>
+      </c>
+      <c r="E23" t="str">
+        <v>AI &amp; Cognitive Systems</v>
+      </c>
+      <c r="F23" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G23" t="str">
+        <v>24 RAG Flow, 08 Component, 09 Data Flow</v>
+      </c>
+      <c r="H23" t="str">
+        <v>18 Trust Boundary, 27 Threat Model, 11 Sequence</v>
+      </c>
+      <c r="I23" t="str">
+        <v>14 Data Model, 25 Tool/Protocol</v>
+      </c>
+      <c r="J23" t="str">
+        <v>GraphRAG (Knowledge Graph Multi-Hop), Hybrid Search (Dense Vector + Sparse BM25), Multimodal RAG (PDF/Images/Audio), Hierarchical RAG</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Vertex AI Vector Search (ScaNN), Cloud Spanner Graph (ISO GQL), Gemini 2.5 Pro / Flash, Document AI, Model Armor</v>
+      </c>
+      <c r="L23" t="str">
+        <v>PRD, FDD, HLD, LLD, AI System Card, Grounding Spec</v>
+      </c>
+      <c r="M23" t="str">
+        <v>OWASP GenAI LLM Top 10 2026, NIST AI RMF 1.0, RAG Triad Standards</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Bio-Pharma Clinical Trials, Enterprise Legal, Customer Support, Internal Knowledge Hubs</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Grounded LLM responses, enterprise document search, hallucination reduction, domain-specific AI querying</v>
+      </c>
+      <c r="P23" t="str">
+        <v>Chunks &amp; Embeds Enterprise Corpus -&gt; Retrieves Top-K Semantically Grounded Chunks -&gt; Prompts Gemini LLM with Factuality Safeguards</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>L1: User query -&gt; Retrieval Engine -&gt; Enterprise Knowledge Base -&gt; Augmented Prompt -&gt; Grounded Response | L2: Document parsing, embedding pipeline, Vector Search + Graph DB, Reranker, Model Armor | L3: ScaNN index parameters, cosine similarity thresholds, ISO GQL multi-hop queries, token budgets</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C24" t="str">
+        <v>AI-02</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Multi-Agent Systems &amp; Orchestration Architecture</v>
+      </c>
+      <c r="E24" t="str">
+        <v>AI &amp; Cognitive Systems</v>
+      </c>
+      <c r="F24" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G24" t="str">
+        <v>23 Agent Interaction, 11 Sequence, 08 Component</v>
+      </c>
+      <c r="H24" t="str">
+        <v>25 Tool/Protocol Interaction, 26 HITL Flow, 12 State Machine</v>
+      </c>
+      <c r="I24" t="str">
+        <v>28 Failure Flow, 30 FinOps Flow</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Hierarchical Supervisor-Subagent, Planner-Executor, Blackboard Architecture, Peer-to-Peer Agent Mesh, Dynamic Swarm</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Vertex AI Agent Engine, LangGraph, CrewAI, AutoGen on GKE Autopilot, Memorystore Redis Session Store</v>
+      </c>
+      <c r="L24" t="str">
+        <v>PRD, FDD, HLD, LLD, Agent Persona Specs, Multi-Agent Protocol Spec</v>
+      </c>
+      <c r="M24" t="str">
+        <v>OWASP GenAI Security Project - Agentic App Security, NIST AI RMF 1.0</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Bio-Pharma Research, Autonomous Coding, Customer Concierge, Financial Advisory</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Complex multi-step reasoning, autonomous task decomposition, multi-agent collaboration</v>
+      </c>
+      <c r="P24" t="str">
+        <v>Decomposes User Intent into Subtasks -&gt; Dispatches to Domain Subagents -&gt; Synthesizes Unified Validated Outcome</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>L1: User -&gt; Supervisor Agent -&gt; Specialized Domain Agents -&gt; Unified Solution | L2: Agent roles, communication bus, shared memory, state machine transitions, tool registry | L3: ReAct prompting loops, reflection loops, maximum recursion limits, JSON schemas, Redis channels</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C25" t="str">
+        <v>AI-03</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Autonomous Agent Tool &amp; Protocol Gateway (MCP / A2A)</v>
+      </c>
+      <c r="E25" t="str">
+        <v>AI &amp; Cognitive Systems</v>
+      </c>
+      <c r="F25" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G25" t="str">
+        <v>25 Tool/Protocol Interaction, 10 Integration, 11 Sequence</v>
+      </c>
+      <c r="H25" t="str">
+        <v>08 Component, 18 Trust Boundary, 27 Threat Model</v>
+      </c>
+      <c r="I25" t="str">
+        <v>12 State Machine, 28 Failure Flow</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Model Context Protocol (MCP) Server/Client, Agent-to-Agent (A2A) Protocol, Function Calling Gateway, OpenAPI Tool Generator</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Model Context Protocol (MCP SDK), Cloud Run MicroVMs, gVisor Sandboxes, BigQuery Tool Server, GitHub MCP Server</v>
+      </c>
+      <c r="L25" t="str">
+        <v>HLD, LLD, Tool Interface Spec (JSON-RPC 2.0 / MCP)</v>
+      </c>
+      <c r="M25" t="str">
+        <v>OWASP GenAI Security Project - Agentic App Security, Least Privilege Tool IAM</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Cross-Industry, Autonomous AI Platforms, Enterprise Automation</v>
+      </c>
+      <c r="O25" t="str">
+        <v>Agent external tool execution, secure standardized API bridging for LLMs, sandboxed code execution</v>
+      </c>
+      <c r="P25" t="str">
+        <v>Exposes Enterprise APIs as MCP Tools -&gt; Authorizes via Zero-Trust Proxy -&gt; Executes in Isolated Sandbox Environment</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>L1: Agent client -&gt; Standard protocol bridge (MCP/A2A) -&gt; Enterprise Tools &amp; Databases | L2: MCP Gateway, tool discovery registry, JSON-RPC 2.0 transport, schema validation, auth interceptor | L3: Stdio/SSE transport streams, tool argument parsing, rate limiting, gVisor container sandboxing</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C26" t="str">
+        <v>AI-04</v>
+      </c>
+      <c r="D26" t="str">
+        <v>AI Safety, Guardrails &amp; Evaluation Architecture</v>
+      </c>
+      <c r="E26" t="str">
+        <v>AI &amp; Cognitive Systems</v>
+      </c>
+      <c r="F26" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G26" t="str">
+        <v>26 HITL Flow, 24 RAG Flow, 21 Observability</v>
+      </c>
+      <c r="H26" t="str">
+        <v>27 Threat Model, 08 Component, 18 Trust Boundary</v>
+      </c>
+      <c r="I26" t="str">
+        <v>11 Sequence, 33 Matrix / Heatmap</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Model Evaluation, Prompt Evaluation, Agent Evaluation, Automated Red Teaming, Runtime Guardrails, Hallucination Prevention</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Vertex AI Gen AI Evaluation Service, Model Armor, Cloud DLP, Cloud Monitoring AI Dashboard</v>
+      </c>
+      <c r="L26" t="str">
+        <v>HLD, LLD, AI Safety &amp; Evaluation Spec, Red Teaming Report</v>
+      </c>
+      <c r="M26" t="str">
+        <v>NIST AI RMF 1.0 (MEASURE/MANAGE), OWASP GenAI LLM Top 10 2026</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Healthcare AI, Financial Advisory AI, Public Sector, Bio-Pharma</v>
+      </c>
+      <c r="O26" t="str">
+        <v>LLM safety guardrails, continuous model evaluation, prompt injection defense, hallucination monitoring</v>
+      </c>
+      <c r="P26" t="str">
+        <v>Evaluates Prompts &amp; Outputs against Safety Policies -&gt; Blocks Toxic/Hallucinatory Content -&gt; Reports to AI Safety Cockpit</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>L1: Input Prompt -&gt; Safety Guardrail Shield -&gt; Model Inference -&gt; Output Verifier -&gt; Human Gate | L2: Model Armor prompt filters, RAG Triad faithfulness scorers, PII tokenizers, real-time alert engine | L3: Evaluation metrics (G-Eval, BERTScore, toxicity thresholds), prompt injection regex rules, latency SLAs</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C27" t="str">
+        <v>AI-05</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Intelligent Document Processing (IDP) Architecture</v>
+      </c>
+      <c r="E27" t="str">
+        <v>AI &amp; Cognitive Systems</v>
+      </c>
+      <c r="F27" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G27" t="str">
+        <v>09 Data Flow, 08 Component, 24 RAG Flow</v>
+      </c>
+      <c r="H27" t="str">
+        <v>01 Context, 26 HITL Flow, 16 Deployment</v>
+      </c>
+      <c r="I27" t="str">
+        <v>11 Sequence, 14 Data Model</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Specialized Form Parser, Multimodal LLM Extraction, Human-in-the-Loop Review Queue, Zero-Shot Document Classifier</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Google Cloud Document AI, Gemini 2.5 Flash Multimodal, Cloud Storage, Cloud Functions, BigQuery</v>
+      </c>
+      <c r="L27" t="str">
+        <v>PRD, FDD, HLD, LLD, Document Schema Definition</v>
+      </c>
+      <c r="M27" t="str">
+        <v>ISO 19005 (PDF/A), HIPAA / SOC 2 Privacy Standards</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Bio-Pharma Clinical Forms, Insurance Claims, Financial Invoices, Legal Contracts</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Unstructured document ingestion, PDF digitization, OCR extraction with validation and HITL routing</v>
+      </c>
+      <c r="P27" t="str">
+        <v>Ingests PDF/Scan Documents -&gt; Extracts Structured Entities via Document AI -&gt; Routes Exceptions to HITL Queue</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>L1: Inbound unstructured docs (PDF, Scans) -&gt; OCR &amp; Extraction -&gt; Validation -&gt; Core ERP/EHR | L2: Document AI processors, confidence threshold routers, HITL review queue, BigQuery schema store | L3: Bounding box coordinate extraction, entity confidence thresholds (e.g. &gt;0.90), webhook dispatchers</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C28" t="str">
+        <v>AI-06</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Logical AI Tenant Isolation &amp; Context Routing</v>
+      </c>
+      <c r="E28" t="str">
+        <v>AI &amp; Cognitive Systems</v>
+      </c>
+      <c r="F28" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G28" t="str">
+        <v>01 Context, 18 Trust Boundary, 08 Component</v>
+      </c>
+      <c r="H28" t="str">
+        <v>17 IAM Flow, 24 RAG Flow, 30 FinOps Flow</v>
+      </c>
+      <c r="I28" t="str">
+        <v>14 Data Model, 25 Tool/Protocol</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Multi-Tenant Prompt Isolation, Tenant Context Propagator, Per-Tenant CMEK Encryption, Tenant Rate &amp; Quota Limiter</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Cloud Run Gateway, Vertex AI Vector Search with Tenant Filters, Cloud Spanner Tenant Tables, Cloud KMS</v>
+      </c>
+      <c r="L28" t="str">
+        <v>HLD, LLD, Multi-Tenant AI Security Spec</v>
+      </c>
+      <c r="M28" t="str">
+        <v>SOC 2 Type II, ISO 27001 Multi-Tenant Isolation</v>
+      </c>
+      <c r="N28" t="str">
+        <v>SaaS AI Copilots, Multi-Tenant Healthcare AI, B2B AI Platforms</v>
+      </c>
+      <c r="O28" t="str">
+        <v>Multi-tenant AI applications, preventing cross-tenant context leakage, tenant-specific model fine-tuning</v>
+      </c>
+      <c r="P28" t="str">
+        <v>Extracts Tenant Identity from Ingress -&gt; Injects Tenant Context &amp; Prompts -&gt; Enforces Tenant KMS &amp; Vector Filters</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>L1: Tenant A/B/C clients -&gt; Context Router -&gt; Isolated AI Processing -&gt; Foundation Models | L2: Cloud Run context gateway, per-tenant prompt templates, vector metadata filters, tenant KMS keys | L3: Tenant JWT claim parsing, ScaNN metadata query filters (`tenant_id == X`), per-tenant token buckets</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C29" t="str">
+        <v>SEC-01</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Enterprise Identity, Access &amp; Zero-Trust Architecture</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Security, Privacy &amp; Sovereignty</v>
+      </c>
+      <c r="F29" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G29" t="str">
+        <v>17 IAM Flow, 18 Trust Boundary, 01 Context</v>
+      </c>
+      <c r="H29" t="str">
+        <v>15 Network Topology, 16 Deployment, 27 Threat Model</v>
+      </c>
+      <c r="I29" t="str">
+        <v>11 Sequence, 21 Observability</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Workload Identity Federation (WIF), BeyondCorp Zero-Trust Context-Aware Access, Multi-Cloud SAML/OIDC SSO, Just-In-Time (JIT) IAM</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Google Cloud Identity, Cloud STS (Security Token Service), IAM Workload Identity Pools, BeyondCorp Enterprise, CyberArk</v>
+      </c>
+      <c r="L29" t="str">
+        <v>HLD, LLD, Enterprise IAM Blueprint, Zero-Trust Access Policy Spec</v>
+      </c>
+      <c r="M29" t="str">
+        <v>NIST SP 800-207 (Zero Trust Architecture), CISA ZT Maturity Model 2.0</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Cross-Industry, Highly Regulated Enterprises, Multi-Cloud</v>
+      </c>
+      <c r="O29" t="str">
+        <v>Multi-cloud identity federation, zero-trust perimeter, eliminating long-lived service account keys</v>
+      </c>
+      <c r="P29" t="str">
+        <v>Authenticates External IdP Tokens -&gt; Exchanges for Short-Lived GCP STS Tokens -&gt; Authorizes Fine-Grained Least-Privilege IAM Roles</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>L1: External Users &amp; IdPs -&gt; Cloud Identity Proxy -&gt; Zero-Trust Policy -&gt; Google Cloud Resources | L2: IdP (Okta/Entra), STS Token Exchange, IAM Workload Identity Pools, Context-Aware Access levels | L3: OIDC claim mapping rules, RFC 8693 token exchange payloads, 1-hour STS session TTLs, conditional IAM</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C30" t="str">
+        <v>SEC-02</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Application &amp; Workload Security Architecture</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Security, Privacy &amp; Sovereignty</v>
+      </c>
+      <c r="F30" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G30" t="str">
+        <v>18 Trust Boundary, 27 Threat Model, 08 Component</v>
+      </c>
+      <c r="H30" t="str">
+        <v>15 Network Topology, 16 Deployment, 21 Observability</v>
+      </c>
+      <c r="I30" t="str">
+        <v>17 IAM Flow, 28 Failure Flow</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Defense-in-Depth AppSec, Software Supply Chain Security (SLSA L3), Cloud Workload Protection (CWPP), API Threat Defense</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Cloud Armor WAF (OWASP rulesets), Cloud KMS (CMEK), Secret Manager, Binary Authorization, Container Analysis, SCC Premium</v>
+      </c>
+      <c r="L30" t="str">
+        <v>HLD, LLD, Threat Model (STRIDE), Security Architecture Review (SAR)</v>
+      </c>
+      <c r="M30" t="str">
+        <v>OWASP Top 10 2021, SLSA Level 3, NIST SP 800-218 (SSDF)</v>
+      </c>
+      <c r="N30" t="str">
+        <v>FinTech, Healthcare, Bio-Pharma, E-Commerce, Government</v>
+      </c>
+      <c r="O30" t="str">
+        <v>Threat modeling, compliance certification (SOC2/PCI/HIPAA), secure software supply chain</v>
+      </c>
+      <c r="P30" t="str">
+        <v>Mitigates Threat Attack Vectors -&gt; Attests Container Signatures via Binary Auth -&gt; Encrypts Data with Customer-Managed Keys (CMEK)</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>L1: External Internet -&gt; Edge WAF -&gt; DMZ Inspection -&gt; Encrypted Workload Enclave -&gt; Secrets Vault | L2: Cloud Armor WAF, Binary Authorization attestor, Secret Manager, Cloud KMS HSM, SCC Premium | L3: WAF rule priorities, Cosign KMS key signatures, envelope encryption AES-GCM 256, runtime syscall audits</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C31" t="str">
+        <v>SEC-03</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Threat Modeling &amp; Attack Surface Architecture (STRIDE)</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Security, Privacy &amp; Sovereignty</v>
+      </c>
+      <c r="F31" t="str">
+        <v>L2, L3</v>
+      </c>
+      <c r="G31" t="str">
+        <v>27 Threat Model, 18 Trust Boundary, 08 Component</v>
+      </c>
+      <c r="H31" t="str">
+        <v>01 Context, 15 Network Topology, 17 IAM Flow</v>
+      </c>
+      <c r="I31" t="str">
+        <v>11 Sequence, 28 Failure Flow</v>
+      </c>
+      <c r="J31" t="str">
+        <v>STRIDE Threat Modeling, Attack Tree Analysis, PASTA Risk-Centric Threat Model, AI Red-Teaming Surface Mapping</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Security Command Center (SCC), Cloud Armor Security Policies, Chronicle SIEM, Model Armor Threat Shield</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Threat Model Document (TMD), Security Architecture Assessment, Penetration Testing Scope</v>
+      </c>
+      <c r="M31" t="str">
+        <v>STRIDE Threat Modeling Standard, NIST SP 800-154, MITRE ATT&amp;CK Framework</v>
+      </c>
+      <c r="N31" t="str">
+        <v>High-Risk Enterprise, Banking, Healthcare, Defense, SaaS</v>
+      </c>
+      <c r="O31" t="str">
+        <v>Formal threat modeling for new architectures, major release security signoff, penetration testing preparation</v>
+      </c>
+      <c r="P31" t="str">
+        <v>Enumerates STRIDE Threat Vectors across Components -&gt; Maps Compensating Controls -&gt; Verifies Mitigation Coverage</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>L1: Threat actors &amp; external attack surfaces | L2: STRIDE threat overlay on system containers &amp; trust boundaries | L3: Detailed exploit paths, CVE vulnerabilities, WAF rule IDs, and cryptographic mitigation proofs</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C32" t="str">
+        <v>SEC-04</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Data Security, Privacy &amp; Sovereign Cloud Architecture</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Security, Privacy &amp; Sovereignty</v>
+      </c>
+      <c r="F32" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G32" t="str">
+        <v>18 Trust Boundary, 34 Geographic Architecture, 09 Data Flow</v>
+      </c>
+      <c r="H32" t="str">
+        <v>14 Data Model, 17 IAM Flow, 21 Observability</v>
+      </c>
+      <c r="I32" t="str">
+        <v>27 Threat Model, 30 FinOps Flow</v>
+      </c>
+      <c r="J32" t="str">
+        <v>EU Sovereign Cloud Boundary, Confidential Computing (AMD SEV), PII De-Identification &amp; Tokenization, External Key Management (EKM)</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Assured Workloads, Cloud KMS with Cloud EKM (Thales/Fortanix), Sensitive Data Protection (DLP), Confidential GKE / VMs</v>
+      </c>
+      <c r="L32" t="str">
+        <v>HLD, LLD, Data Privacy Impact Assessment (DPIA), Sovereign Cloud Compliance Pack</v>
+      </c>
+      <c r="M32" t="str">
+        <v>EU GDPR, HIPAA Security Rule, FedRAMP High, BSI C5 (Germany)</v>
+      </c>
+      <c r="N32" t="str">
+        <v>European Enterprises, Healthcare &amp; Genomics, Public Sector, Defense</v>
+      </c>
+      <c r="O32" t="str">
+        <v>Cross-border data regulations, sovereign cloud boundaries, strict data residency requirements</v>
+      </c>
+      <c r="P32" t="str">
+        <v>Enforces Sovereign Boundary Controls -&gt; Protects Data-in-Use via Confidential Hardware Enclaves -&gt; Anonymizes PII via DLP</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>L1: Geographic jurisdictions (EU/US/APAC) -&gt; Sovereign Landing Zones -&gt; Local Key Custody -&gt; Regulated Users | L2: Assured Workloads EU boundary, Cloud EKM local HSM, DLP tokenization pipeline, Confidential GKE nodes | L3: AMD SEV hardware memory encryption keys, DLP regex/surrogate rules, regional bucket replication limits</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="C33" t="str">
+        <v>OPS-01</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Enterprise Observability, Telemetry &amp; SRE Architecture</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Operations &amp; SRE</v>
+      </c>
+      <c r="F33" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G33" t="str">
+        <v>21 Observability / SRE, 08 Component, 07 Container</v>
+      </c>
+      <c r="H33" t="str">
+        <v>16 Deployment, 28 Failure Flow, 29 Cutover Runbook</v>
+      </c>
+      <c r="I33" t="str">
+        <v>11 Sequence, 30 FinOps Flow</v>
+      </c>
+      <c r="J33" t="str">
+        <v>OpenTelemetry Unified Observability, SLO/Error Budget Driven Operations, Centralized Log Aggregation &amp; SIEM, Distributed APM Tracing</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Google Cloud Logging, Cloud Monitoring, Cloud Trace, Cloud Profiler, OpenTelemetry Collector, Managed Prometheus</v>
+      </c>
+      <c r="L33" t="str">
+        <v>HLD, LLD, SRE Runbook, SLO / SLA Definition Document</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Google SRE Principles, OpenTelemetry 1.0 Standard, ISO 20000</v>
+      </c>
+      <c r="N33" t="str">
+        <v>Cross-Industry, Mission-Critical Systems, 24/7 Operations</v>
+      </c>
+      <c r="O33" t="str">
+        <v>Production reliability engineering, SLO monitoring, distributed microservice tracing, proactive incident management</v>
+      </c>
+      <c r="P33" t="str">
+        <v>Collects Metrics/Logs/Traces from All Workloads -&gt; Evaluates SLO Burn Rates -&gt; Dispatches Automated PagerDuty &amp; Self-Healing Actions</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>L1: Workload telemetry producers -&gt; Central Observability Pipeline -&gt; Real-Time SRE Cockpit -&gt; Incident Response | L2: OpenTelemetry sidecars, Cloud Logging log router, Managed Prometheus collectors, Grafana, PagerDuty | L3: PromQL alert expressions, SLO error budget burn rate algorithms, trace sampling filters (10%), metric sinks</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Operational</v>
+      </c>
+      <c r="C34" t="str">
+        <v>OPS-02</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Operational Readiness &amp; Go-Live Cutover Runbook</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Operations &amp; SRE</v>
+      </c>
+      <c r="F34" t="str">
+        <v>L2, L3</v>
+      </c>
+      <c r="G34" t="str">
+        <v>29 Cutover Runbook, 03 Swimlane, 11 Sequence</v>
+      </c>
+      <c r="H34" t="str">
+        <v>28 Failure Flow, 21 Observability, 19 HA/DR</v>
+      </c>
+      <c r="I34" t="str">
+        <v>32 Timeline / Roadmap</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Phased Cutover (Wave-by-Wave), Big-Bang Maintenance Window, Dark Launch with Shadow Traffic, Live Zero-Downtime Migration</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Cloud Logging War Room Dashboard, Cloud Deploy Canary Targets, Datastream CDC Sync, PagerDuty Event Bridge</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Go-Live Runbook, Cutover Checklist, Rollback Protocol, Production Readiness Review (PRR)</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Google Production Readiness Review (PRR) Standard</v>
+      </c>
+      <c r="N34" t="str">
+        <v>Mission-Critical Launches, Core Banking Cutover, EHR Migration</v>
+      </c>
+      <c r="O34" t="str">
+        <v>Production release cutover, major datacenter-to-cloud migration go-live, BCDR disaster simulation</v>
+      </c>
+      <c r="P34" t="str">
+        <v>Executes Step-by-Step Cutover Checklist -&gt; Monitors Real-Time War Room Health Checks -&gt; Triggers Rollback if Smoke Tests Fail</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>L1: Pre-Cutover Verification -&gt; Maintenance Window -&gt; Data Freeze &amp; Final Sync -&gt; Cutover -&gt; Signoff | L2: War Room command chain, synchronization checks, DNS switchover, validation smoke suites, rollback matrix | L3: Minute-by-minute execution steps (T-120 to T+60), exact gcloud CLI cutover commands, automated health checks</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Operational</v>
+      </c>
+      <c r="C35" t="str">
+        <v>STR-01</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Enterprise Discovery, Assessment &amp; Migration Waves</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Strategic &amp; Operating Models</v>
+      </c>
+      <c r="F35" t="str">
+        <v>L1, L2</v>
+      </c>
+      <c r="G35" t="str">
+        <v>05 As-Is / To-Be, 04 Value Stream, 31 Dependency Map</v>
+      </c>
+      <c r="H35" t="str">
+        <v>32 Timeline / Roadmap, 02 Capability Map, 30 FinOps Flow</v>
+      </c>
+      <c r="I35" t="str">
+        <v>33 Matrix / Heatmap</v>
+      </c>
+      <c r="J35" t="str">
+        <v>6-Rs Migration Strategy (Rehost, Replatform, Refactor, Repurchase, Retain, Retire), Factory Wave Migration</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Google Cloud Migration Center, StrataZone, Carbon Footprint Analyzer, BigQuery Dependency Graph</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Migration Assessment Report, Total Cost of Ownership (TCO) Study, Wave Migration Master Plan</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Google Cloud Architecture Framework - System Design &amp; Migration</v>
+      </c>
+      <c r="N35" t="str">
+        <v>Datacenter Modernization, Legacy Transformation</v>
+      </c>
+      <c r="O35" t="str">
+        <v>Datacenter exit, hardware refresh cycle, enterprise cloud transformation initiative</v>
+      </c>
+      <c r="P35" t="str">
+        <v>Discovers Legacy Asset Inventory -&gt; Maps Inter-Application Dependencies -&gt; Categorizes into 6-Rs Migration Waves</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>L1: Legacy Silos -&gt; Automated Discovery &amp; Mapping -&gt; Migration Wave Planning -&gt; Target Cloud Architecture | L2: Migration Center collectors, dependency clustering algorithms, wave prioritization matrix (Wave 1/2/3), TCO | L3: Server inventory schemas, network port dependency maps, wave execution timelines, migration risk scoring</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Operational</v>
+      </c>
+      <c r="C36" t="str">
+        <v>STR-02</v>
+      </c>
+      <c r="D36" t="str">
+        <v>AI Operating Model, Governance &amp; Decision Framework</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Strategic &amp; Operating Models</v>
+      </c>
+      <c r="F36" t="str">
+        <v>L1, L2</v>
+      </c>
+      <c r="G36" t="str">
+        <v>02 Capability Map, 26 HITL Flow, 04 Value Stream</v>
+      </c>
+      <c r="H36" t="str">
+        <v>03 Swimlane, 33 Matrix / Heatmap, 27 Threat Model</v>
+      </c>
+      <c r="I36" t="str">
+        <v>31 Dependency Map</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Centralized AI Center of Excellence (CoE), Hub-and-Spoke Federated AI Teams, Autonomous Product Pods with Safety Gate</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Vertex AI Model Evaluation, Model Armor, Vertex AI Gen AI Evaluation Service, Jira Enterprise, ServiceNow</v>
+      </c>
+      <c r="L36" t="str">
+        <v>AI Operating Model Strategy, AI Ethics Charter, Model Governance Framework</v>
+      </c>
+      <c r="M36" t="str">
+        <v>NIST AI RMF 1.0 (GOVERN/MAP/MEASURE/MANAGE), EU AI Act (High-Risk)</v>
+      </c>
+      <c r="N36" t="str">
+        <v>Enterprise AI Strategy, Healthcare AI, Financial Services AI</v>
+      </c>
+      <c r="O36" t="str">
+        <v>Enterprise AI adoption, regulatory compliance for LLMs, establishing AI safety &amp; ethics committee</v>
+      </c>
+      <c r="P36" t="str">
+        <v>Defines AI Governance Policies -&gt; Validates Model Safety Metrics via Evaluation Suites -&gt; Grants Production Release Approval</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>L1: Enterprise AI Strategy -&gt; Use Case Intake &amp; Risk Triage -&gt; AI Ethics Board -&gt; Operationalization | L2: AI CoE steering committee, model validation workflow, prompt red-teaming board, compliance monitoring | L3: Evaluation thresholds (faithfulness &gt; 0.95, toxicity = 0), human review escalation criteria, RACI matrix</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Operational</v>
+      </c>
+      <c r="C37" t="str">
+        <v>STR-03</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Cloud FinOps &amp; Automated Cost Governance</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Strategic &amp; Operating Models</v>
+      </c>
+      <c r="F37" t="str">
+        <v>L1, L2</v>
+      </c>
+      <c r="G37" t="str">
+        <v>30 FinOps Flow, 02 Capability Map, 04 Value Stream</v>
+      </c>
+      <c r="H37" t="str">
+        <v>09 Data Flow, 33 Matrix / Heatmap, 31 Dependency Map</v>
+      </c>
+      <c r="I37" t="str">
+        <v>28 Failure Flow</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Unit Economics Cost Allocation, Automated Idle Resource Reclaimer, Shared Infrastructure Chargeback, AI Token Cost Attribution</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Google Cloud Billing BigQuery Export, Looker FinOps Studio, Dataform SQLX, Active Assist Recommendations, Cloud Functions</v>
+      </c>
+      <c r="L37" t="str">
+        <v>FinOps Operating Framework, Cloud Cost Allocation Policy, Executive Budget Plan</v>
+      </c>
+      <c r="M37" t="str">
+        <v>FinOps Foundation Framework (Inform / Optimize / Operate)</v>
+      </c>
+      <c r="N37" t="str">
+        <v>Cross-Industry, Enterprise Cloud Economics</v>
+      </c>
+      <c r="O37" t="str">
+        <v>Cloud cost transparency, shared cost attribution, reducing cloud waste, AI GPU/token budgeting</v>
+      </c>
+      <c r="P37" t="str">
+        <v>Exports Detailed Billing Telemetry -&gt; Allocates Costs by Business Unit &amp; App Labels -&gt; Automates Idle Reclaim &amp; Executive Billing</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>L1: Cloud Usage Telemetry -&gt; FinOps Ingestion -&gt; Cost Attribution Marts -&gt; Executive Dashboards &amp; Optimization | L2: Cloud Billing export, Dataform transformation jobs, BigQuery FinOps dataset, Looker dashboards, Active Assist | L3: Label inheritance hierarchies, shared GKE cluster cost distribution formulas, budget alert webhooks</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Industry Accelerator</v>
+      </c>
+      <c r="C38" t="str">
+        <v>IND-01</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Bio-Pharma Precision Oncology &amp; Regulatory Platform</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Industry Accelerators</v>
+      </c>
+      <c r="F38" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G38" t="str">
+        <v>01 Context, 09 Data Flow, 24 RAG Flow, 18 Trust Boundary</v>
+      </c>
+      <c r="H38" t="str">
+        <v>23 Agent Interaction, 26 HITL Flow, 34 Geographic</v>
+      </c>
+      <c r="I38" t="str">
+        <v>14 Data Model, 27 Threat Model</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Genomic Sequencing Pipeline, Clinical Trial Regulatory Intelligence, Molecular Drug Discovery RAG, Patient Cohort Explorer</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Google Cloud Life Sciences API, Vertex AI Gemini 2.5 Pro, Cloud Spanner Graph (ISO GQL), Dataplex Life Sciences Mesh, Assured Workloads</v>
+      </c>
+      <c r="L38" t="str">
+        <v>PRD, FDD, HLD, LLD, 21 CFR Part 11 Validation Pack, HIPAA Compliance Audit</v>
+      </c>
+      <c r="M38" t="str">
+        <v>FDA 21 CFR Part 11, HIPAA Security Rule, GxP Computerized Systems Validation (CSV), GAMP 5</v>
+      </c>
+      <c r="N38" t="str">
+        <v>Bio-Pharma, Genomics, Precision Oncology, Clinical Trials, Regulatory Affairs</v>
+      </c>
+      <c r="O38" t="str">
+        <v>Next-Gen Sequencing (NGS) data processing, FDA regulatory document automation, multi-hop biomedical knowledge graphs</v>
+      </c>
+      <c r="P38" t="str">
+        <v>Composes Data Lakehouse + RAG + Multi-Agent + GxP Zero Trust -&gt; Accelerated Clinical Insights with 100% Audit Immutability</v>
+      </c>
+      <c r="Q38" t="str">
+        <v>L1: Genomic Sequencers &amp; EHRs -&gt; Biomedical Knowledge -&gt; Genomic Variant AI -&gt; Clinical Trials -&gt; FDA Submissions | L2: FASTQ/BAM ingestion pipelines, Spanner ISO GQL Genomic Knowledge Graph, Vertex RAG, Model Armor | L3: GxP immutable audit trails, electronic signatures (21 CFR Part 11), ScaNN embeddings of PubMed, HIPAA encryption</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Industry Accelerator</v>
+      </c>
+      <c r="C39" t="str">
+        <v>IND-02</v>
+      </c>
+      <c r="D39" t="str">
+        <v>FinTech Autonomous Wealth &amp; Financial Fraud Engine</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Industry Accelerators</v>
+      </c>
+      <c r="F39" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G39" t="str">
+        <v>01 Context, 09 Data Flow, 11 Sequence, 18 Trust Boundary</v>
+      </c>
+      <c r="H39" t="str">
+        <v>10 Integration, 27 Threat Model, 30 FinOps Flow</v>
+      </c>
+      <c r="I39" t="str">
+        <v>12 State Machine, 28 Failure Flow</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Personalized Robo-Advisory, Real-Time Transaction Fraud Detection, Algorithmic Risk Assessment, Open Banking API Platform</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Cloud Spanner Multi-Region TrueTime, BigQuery Continuous Queries, Cloud Dataflow Streaming, Apigee X Banking APIs, Vertex AI Fraud</v>
+      </c>
+      <c r="L39" t="str">
+        <v>PRD, FDD, HLD, LLD, PCI-DSS Attestation of Compliance (AoC), Model Risk Management (SR 11-7)</v>
+      </c>
+      <c r="M39" t="str">
+        <v>PCI-DSS v4.0, Federal Reserve SR 11-7 Model Risk Management, FFIEC IT Handbook</v>
+      </c>
+      <c r="N39" t="str">
+        <v>FinTech, Retail Banking, Wealth Management, Payments, Fraud Prevention</v>
+      </c>
+      <c r="O39" t="str">
+        <v>Sub-millisecond payment authorization, real-time AML/fraud scoring, personalized portfolio optimization</v>
+      </c>
+      <c r="P39" t="str">
+        <v>Composes Real-Time Streaming + Spanner TrueTime + Apigee X Banking Gateway -&gt; Ultra-low latency financial transactions with PCI compliance</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>L1: Banking Clients -&gt; Open Banking Gateway -&gt; Real-Time Fraud &amp; Wealth AI -&gt; Core Ledger -&gt; Market Execution | L2: Apigee X PCI gateway, Dataflow sub-second stream analytics, Cloud Spanner multi-region ledger, Vertex AI | L3: ISO 20022 message schemas, TrueTime external consistency guarantees, HSM payment tokenization</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Industry Accelerator</v>
+      </c>
+      <c r="C40" t="str">
+        <v>IND-03</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Smart Manufacturing &amp; Industrial IoT Predictive Maintenance</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Industry Accelerators</v>
+      </c>
+      <c r="F40" t="str">
+        <v>L1, L2, L3</v>
+      </c>
+      <c r="G40" t="str">
+        <v>01 Context, 09 Data Flow, 15 Network Topology, 16 Deployment</v>
+      </c>
+      <c r="H40" t="str">
+        <v>08 Component, 21 Observability, 28 Failure Flow</v>
+      </c>
+      <c r="I40" t="str">
+        <v>12 State Machine, 34 Geographic</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Edge AI Anomaly Detection, Factory Digital Twin, Supply Chain Real-Time Telemetry, Automated Quality Visual Inspection</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Google Distributed Cloud (GDC) Edge, Cloud Pub/Sub, Dataflow, BigQuery IoT Data Marts, Vertex AI Vision, Looker Industrial Ops</v>
+      </c>
+      <c r="L40" t="str">
+        <v>PRD, FDD, HLD, LLD, Factory OT/IT Integration Spec, ISA-95 Architecture Doc</v>
+      </c>
+      <c r="M40" t="str">
+        <v>ISA-95 Enterprise-Control Integration, IEC 62443 Industrial Cybersecurity, ISO 9001</v>
+      </c>
+      <c r="N40" t="str">
+        <v>Manufacturing, Industrial IoT, Smart Factories, Automotive, Energy &amp; Utilities</v>
+      </c>
+      <c r="O40" t="str">
+        <v>Factory floor sensor telemetry, industrial machine predictive maintenance, edge computer vision quality control</v>
+      </c>
+      <c r="P40" t="str">
+        <v>Composes Edge Computing + IoT Ingestion + Streaming Anomaly Detection + Digital Twin -&gt; Zero Unplanned Factory Downtime</v>
+      </c>
+      <c r="Q40" t="str">
+        <v>L1: Factory OT Sensors &amp; PLC Controllers -&gt; GDC Edge Gateways -&gt; Cloud IoT Ingestion -&gt; Predictive AI -&gt; Factory HMI | L2: MQTT/OPC-UA edge brokers, GDC Edge clusters, Pub/Sub ingestion, BigQuery time-series datasets, Looker | L3: Vibration FFT spectrum anomaly detection models, edge inference latency budgets (&lt;10ms), Modbus protocol adapters</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q40"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F35"/>
   <sheetData>
     <row r="1">
@@ -3241,7 +5373,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D9"/>
   <sheetData>
@@ -3378,7 +5510,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E17"/>
   <sheetData>
@@ -3678,7 +5810,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F7"/>
   <sheetData>

</xml_diff>